<commit_message>
Re-base PVA model on confirmed demand: 1300 lb/week
Demand confirmed at ~1,300 lb finished liquid/week (~2.9 drums/wk,
~150 drums/yr, ~$50.7k/yr all-SNP). Switched primary input to lb/week
(how SNP bills) and re-derived drums. Resolves the prior 55-vs-220 gal
ambiguity.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkE2ZRYs3PLyj8XHTsU3i4
</commit_message>
<xml_diff>
--- a/PVA_Second_Source_Pricing_Model.xlsx
+++ b/PVA_Second_Source_Pricing_Model.xlsx
@@ -17,17 +17,18 @@
     <definedName name="DrumGal">'Inputs &amp; Assumptions'!$C$6</definedName>
     <definedName name="DrumLb">'Inputs &amp; Assumptions'!$C$7</definedName>
     <definedName name="WeeksYr">'Inputs &amp; Assumptions'!$C$8</definedName>
-    <definedName name="DrumsWk">'Inputs &amp; Assumptions'!$C$9</definedName>
+    <definedName name="DemandLbWk">'Inputs &amp; Assumptions'!$C$9</definedName>
     <definedName name="SNPlb">'Inputs &amp; Assumptions'!$C$10</definedName>
     <definedName name="SNPdrum">'Inputs &amp; Assumptions'!$C$11</definedName>
-    <definedName name="DrumsYr">'Inputs &amp; Assumptions'!$C$12</definedName>
-    <definedName name="GalYr">'Inputs &amp; Assumptions'!$C$13</definedName>
-    <definedName name="BaselineSpend">'Inputs &amp; Assumptions'!$C$14</definedName>
-    <definedName name="APVminGal">'Inputs &amp; Assumptions'!$C$17</definedName>
-    <definedName name="APVlow">'Inputs &amp; Assumptions'!$C$18</definedName>
-    <definedName name="APVlikely">'Inputs &amp; Assumptions'!$C$19</definedName>
-    <definedName name="APVhigh">'Inputs &amp; Assumptions'!$C$20</definedName>
-    <definedName name="SNPsurch">'Inputs &amp; Assumptions'!$C$23</definedName>
+    <definedName name="DrumsWk">'Inputs &amp; Assumptions'!$C$12</definedName>
+    <definedName name="DrumsYr">'Inputs &amp; Assumptions'!$C$13</definedName>
+    <definedName name="GalYr">'Inputs &amp; Assumptions'!$C$14</definedName>
+    <definedName name="BaselineSpend">'Inputs &amp; Assumptions'!$C$15</definedName>
+    <definedName name="APVminGal">'Inputs &amp; Assumptions'!$C$18</definedName>
+    <definedName name="APVlow">'Inputs &amp; Assumptions'!$C$19</definedName>
+    <definedName name="APVlikely">'Inputs &amp; Assumptions'!$C$20</definedName>
+    <definedName name="APVhigh">'Inputs &amp; Assumptions'!$C$21</definedName>
+    <definedName name="SNPsurch">'Inputs &amp; Assumptions'!$C$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -36,9 +37,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="165" formatCode="$0.00"/>
-    <numFmt numFmtId="166" formatCode="$#,##0"/>
+    <numFmt numFmtId="164" formatCode="$0.00"/>
+    <numFmt numFmtId="165" formatCode="$#,##0"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
   <fonts count="8">
@@ -155,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -169,24 +170,27 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="9" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -199,24 +203,24 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="166" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="167" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -227,7 +231,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -605,7 +609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E31"/>
+  <dimension ref="B2:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -681,15 +685,15 @@
     <row r="9">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>TOTAL demand (drums / week)  &lt;-- KEY INPUT</t>
+          <t>TOTAL demand (lb finished PVA / week)  &lt;-- KEY INPUT</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>1</v>
+        <v>1300</v>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>DISCREPANCY: Notion RFQ says ~4 drums/wk (220 gal). Recent APV framing says ~1 drum/wk (55 gal) TOTAL. Flip this to test both.</t>
+          <t>Confirmed by Oscar 2026-06-26: ~1,300 lb finished liquid/wk. This is how SNP bills (per lb). Supersedes the old 55 vs 220 gal estimates.</t>
         </is>
       </c>
     </row>
@@ -726,181 +730,196 @@
     <row r="12">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Total drums per year</t>
+          <t>Total demand (drums / week)</t>
         </is>
       </c>
       <c r="C12" s="10">
-        <f>DrumsWk*WeeksYr</f>
+        <f>DemandLbWk/DrumLb</f>
+        <v/>
+      </c>
+      <c r="E12" s="6">
+        <f> lb/wk / drum lb</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Total gallons per year</t>
+          <t>Total drums per year</t>
         </is>
       </c>
       <c r="C13" s="11">
-        <f>DrumsYr*DrumGal</f>
+        <f>DrumsWk*WeeksYr</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="4" t="inlineStr">
         <is>
+          <t>Total gallons per year</t>
+        </is>
+      </c>
+      <c r="C14" s="12">
+        <f>DrumsYr*DrumGal</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
           <t>CURRENT all-SNP annual spend ($)</t>
         </is>
       </c>
-      <c r="C14" s="9">
+      <c r="C15" s="9">
         <f>DrumsYr*SNPdrum</f>
         <v/>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>Baseline: 100% to SNP.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="3" t="inlineStr">
+    <row r="17">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>2) APV / SECOND-SOURCE PRICE ASSUMPTIONS (placeholders until real quote)</t>
         </is>
       </c>
-      <c r="C16" s="3" t="n"/>
-      <c r="D16" s="3" t="n"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>APV minimum batch (gallons)</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>APV Engineered Coatings advertises 100-8,700 gal batches. A single 55-gal drum is BELOW min -&gt; order in 2-drum (110 gal) runs to be efficient.</t>
-        </is>
-      </c>
+      <c r="C17" s="3" t="n"/>
+      <c r="D17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>APV price/drum - LOW (best case)</t>
-        </is>
-      </c>
-      <c r="C18" s="12">
-        <f>SNPdrum</f>
-        <v/>
+          <t>APV minimum batch (gallons)</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Parity with SNP. Unlikely at low volume; optimistic floor.</t>
+          <t>APV Engineered Coatings advertises 100-8,700 gal batches. A single 55-gal drum is BELOW min -&gt; order in 2-drum (110 gal) runs to be efficient.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>APV price/drum - LIKELY</t>
-        </is>
-      </c>
-      <c r="C19" s="12">
-        <f>ROUND(SNPdrum*1.5,2)</f>
+          <t>APV price/drum - LOW (best case)</t>
+        </is>
+      </c>
+      <c r="C19" s="13">
+        <f>SNPdrum</f>
         <v/>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>+50% small-batch premium. ADJUST when APV quotes.</t>
+          <t>Parity with SNP. Unlikely at low volume; optimistic floor.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="4" t="inlineStr">
         <is>
+          <t>APV price/drum - LIKELY</t>
+        </is>
+      </c>
+      <c r="C20" s="13">
+        <f>ROUND(SNPdrum*1.5,2)</f>
+        <v/>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>+50% small-batch premium. ADJUST when APV quotes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="4" t="inlineStr">
+        <is>
           <t>APV price/drum - HIGH (single-drum penalty)</t>
         </is>
       </c>
-      <c r="C20" s="12">
+      <c r="C21" s="13">
         <f>ROUND(SNPdrum*2,2)</f>
         <v/>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>+100%: pays for ~100-gal min batch to make one drum.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="3" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>3) SNP RE-PRICING RISK (if SNP loses volume to a 2nd source)</t>
         </is>
       </c>
-      <c r="C22" s="3" t="n"/>
-      <c r="D22" s="3" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="4" t="inlineStr">
+      <c r="C23" s="3" t="n"/>
+      <c r="D23" s="3" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>SNP surcharge if volume reduced (%)</t>
         </is>
       </c>
-      <c r="C23" s="13" t="n">
+      <c r="C24" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr">
         <is>
           <t>Set e.g. 10% to test: does SNP raise the rate on remaining drums once they lose the full account? Used in scenarios.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="14" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="15" t="inlineStr">
         <is>
           <t>HOW TO USE:</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Tab 'Split Scenarios': compare giving APV 0/10/20/25/33/50% of volume at the LIKELY price.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Tab 'APV Price Sensitivity': how total cost moves with APV's real quote x the split.</t>
+          <t xml:space="preserve">  - Tab 'Split Scenarios': compare giving APV 0/10/20/25/33/50% of volume at the LIKELY price.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Tab 'SNP Re-pricing Risk': the breakeven - how big an SNP surcharge erases the value of a 2nd source.</t>
+          <t xml:space="preserve">  - Tab 'APV Price Sensitivity': how total cost moves with APV's real quote x the split.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Tab 'Supplier Capacity': who is big/small and whether a single-drum account fits them.</t>
+          <t xml:space="preserve">  - Tab 'SNP Re-pricing Risk': the breakeven - how big an SNP surcharge erases the value of a 2nd source.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>DECIDED: fixed split ~20-25% to APV (~quote per drum, recurring rotation). Highlighted in Split Scenarios.</t>
+          <t xml:space="preserve">  - Tab 'Supplier Capacity': who is big/small and whether a single-drum account fits them.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>DECIDED: fixed split ~20-25% to APV (~quote per drum, recurring rotation). Highlighted in Split Scenarios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>REMEMBER: real viscosity target is still pending from SNP CoA history - APV cannot finalize a firm quote without it.</t>
         </is>
@@ -947,301 +966,301 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>Split % to APV</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>APV drums/yr</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>SNP drums/yr</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="D4" s="16" t="inlineStr">
         <is>
           <t>SNP $/drum
 (w/ surcharge)</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>APV $/drum
 (Likely)</t>
         </is>
       </c>
-      <c r="F4" s="15" t="inlineStr">
+      <c r="F4" s="16" t="inlineStr">
         <is>
           <t>SNP annual $</t>
         </is>
       </c>
-      <c r="G4" s="15" t="inlineStr">
+      <c r="G4" s="16" t="inlineStr">
         <is>
           <t>APV annual $</t>
         </is>
       </c>
-      <c r="H4" s="15" t="inlineStr">
+      <c r="H4" s="16" t="inlineStr">
         <is>
           <t>TOTAL annual $</t>
         </is>
       </c>
-      <c r="I4" s="15" t="inlineStr">
+      <c r="I4" s="16" t="inlineStr">
         <is>
           <t>Δ vs all-SNP $</t>
         </is>
       </c>
-      <c r="J4" s="15" t="inlineStr">
+      <c r="J4" s="16" t="inlineStr">
         <is>
           <t>Δ %</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="n">
+      <c r="A5" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="B5" s="17">
+      <c r="B5" s="18">
         <f>ROUND(DrumsYr*A5,1)</f>
         <v/>
       </c>
-      <c r="C5" s="17">
+      <c r="C5" s="18">
         <f>ROUND(DrumsYr*(1-A5),1)</f>
         <v/>
       </c>
-      <c r="D5" s="18">
+      <c r="D5" s="19">
         <f>IF(A5&gt;0,SNPdrum*(1+SNPsurch),SNPdrum)</f>
         <v/>
       </c>
-      <c r="E5" s="18">
+      <c r="E5" s="19">
         <f>APVlikely</f>
         <v/>
       </c>
-      <c r="F5" s="18">
+      <c r="F5" s="19">
         <f>C5*D5</f>
         <v/>
       </c>
-      <c r="G5" s="18">
+      <c r="G5" s="19">
         <f>B5*E5</f>
         <v/>
       </c>
-      <c r="H5" s="18">
+      <c r="H5" s="19">
         <f>F5+G5</f>
         <v/>
       </c>
-      <c r="I5" s="18">
+      <c r="I5" s="19">
         <f>H5-BaselineSpend</f>
         <v/>
       </c>
-      <c r="J5" s="19">
+      <c r="J5" s="20">
         <f>IF(BaselineSpend=0,0,I5/BaselineSpend)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="n">
+      <c r="A6" s="17" t="n">
         <v>0.1</v>
       </c>
-      <c r="B6" s="17">
+      <c r="B6" s="18">
         <f>ROUND(DrumsYr*A6,1)</f>
         <v/>
       </c>
-      <c r="C6" s="17">
+      <c r="C6" s="18">
         <f>ROUND(DrumsYr*(1-A6),1)</f>
         <v/>
       </c>
-      <c r="D6" s="18">
+      <c r="D6" s="19">
         <f>IF(A6&gt;0,SNPdrum*(1+SNPsurch),SNPdrum)</f>
         <v/>
       </c>
-      <c r="E6" s="18">
+      <c r="E6" s="19">
         <f>APVlikely</f>
         <v/>
       </c>
-      <c r="F6" s="18">
+      <c r="F6" s="19">
         <f>C6*D6</f>
         <v/>
       </c>
-      <c r="G6" s="18">
+      <c r="G6" s="19">
         <f>B6*E6</f>
         <v/>
       </c>
-      <c r="H6" s="18">
+      <c r="H6" s="19">
         <f>F6+G6</f>
         <v/>
       </c>
-      <c r="I6" s="18">
+      <c r="I6" s="19">
         <f>H6-BaselineSpend</f>
         <v/>
       </c>
-      <c r="J6" s="19">
+      <c r="J6" s="20">
         <f>IF(BaselineSpend=0,0,I6/BaselineSpend)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="n">
+      <c r="A7" s="21" t="n">
         <v>0.2</v>
       </c>
-      <c r="B7" s="21">
+      <c r="B7" s="22">
         <f>ROUND(DrumsYr*A7,1)</f>
         <v/>
       </c>
-      <c r="C7" s="21">
+      <c r="C7" s="22">
         <f>ROUND(DrumsYr*(1-A7),1)</f>
         <v/>
       </c>
-      <c r="D7" s="22">
+      <c r="D7" s="23">
         <f>IF(A7&gt;0,SNPdrum*(1+SNPsurch),SNPdrum)</f>
         <v/>
       </c>
-      <c r="E7" s="22">
+      <c r="E7" s="23">
         <f>APVlikely</f>
         <v/>
       </c>
-      <c r="F7" s="22">
+      <c r="F7" s="23">
         <f>C7*D7</f>
         <v/>
       </c>
-      <c r="G7" s="22">
+      <c r="G7" s="23">
         <f>B7*E7</f>
         <v/>
       </c>
-      <c r="H7" s="22">
+      <c r="H7" s="23">
         <f>F7+G7</f>
         <v/>
       </c>
-      <c r="I7" s="22">
+      <c r="I7" s="23">
         <f>H7-BaselineSpend</f>
         <v/>
       </c>
-      <c r="J7" s="23">
+      <c r="J7" s="24">
         <f>IF(BaselineSpend=0,0,I7/BaselineSpend)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="n">
+      <c r="A8" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="B8" s="21">
+      <c r="B8" s="22">
         <f>ROUND(DrumsYr*A8,1)</f>
         <v/>
       </c>
-      <c r="C8" s="21">
+      <c r="C8" s="22">
         <f>ROUND(DrumsYr*(1-A8),1)</f>
         <v/>
       </c>
-      <c r="D8" s="22">
+      <c r="D8" s="23">
         <f>IF(A8&gt;0,SNPdrum*(1+SNPsurch),SNPdrum)</f>
         <v/>
       </c>
-      <c r="E8" s="22">
+      <c r="E8" s="23">
         <f>APVlikely</f>
         <v/>
       </c>
-      <c r="F8" s="22">
+      <c r="F8" s="23">
         <f>C8*D8</f>
         <v/>
       </c>
-      <c r="G8" s="22">
+      <c r="G8" s="23">
         <f>B8*E8</f>
         <v/>
       </c>
-      <c r="H8" s="22">
+      <c r="H8" s="23">
         <f>F8+G8</f>
         <v/>
       </c>
-      <c r="I8" s="22">
+      <c r="I8" s="23">
         <f>H8-BaselineSpend</f>
         <v/>
       </c>
-      <c r="J8" s="23">
+      <c r="J8" s="24">
         <f>IF(BaselineSpend=0,0,I8/BaselineSpend)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="n">
+      <c r="A9" s="17" t="n">
         <v>0.33</v>
       </c>
-      <c r="B9" s="17">
+      <c r="B9" s="18">
         <f>ROUND(DrumsYr*A9,1)</f>
         <v/>
       </c>
-      <c r="C9" s="17">
+      <c r="C9" s="18">
         <f>ROUND(DrumsYr*(1-A9),1)</f>
         <v/>
       </c>
-      <c r="D9" s="18">
+      <c r="D9" s="19">
         <f>IF(A9&gt;0,SNPdrum*(1+SNPsurch),SNPdrum)</f>
         <v/>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="19">
         <f>APVlikely</f>
         <v/>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="19">
         <f>C9*D9</f>
         <v/>
       </c>
-      <c r="G9" s="18">
+      <c r="G9" s="19">
         <f>B9*E9</f>
         <v/>
       </c>
-      <c r="H9" s="18">
+      <c r="H9" s="19">
         <f>F9+G9</f>
         <v/>
       </c>
-      <c r="I9" s="18">
+      <c r="I9" s="19">
         <f>H9-BaselineSpend</f>
         <v/>
       </c>
-      <c r="J9" s="19">
+      <c r="J9" s="20">
         <f>IF(BaselineSpend=0,0,I9/BaselineSpend)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="n">
+      <c r="A10" s="17" t="n">
         <v>0.5</v>
       </c>
-      <c r="B10" s="17">
+      <c r="B10" s="18">
         <f>ROUND(DrumsYr*A10,1)</f>
         <v/>
       </c>
-      <c r="C10" s="17">
+      <c r="C10" s="18">
         <f>ROUND(DrumsYr*(1-A10),1)</f>
         <v/>
       </c>
-      <c r="D10" s="18">
+      <c r="D10" s="19">
         <f>IF(A10&gt;0,SNPdrum*(1+SNPsurch),SNPdrum)</f>
         <v/>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="19">
         <f>APVlikely</f>
         <v/>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="19">
         <f>C10*D10</f>
         <v/>
       </c>
-      <c r="G10" s="18">
+      <c r="G10" s="19">
         <f>B10*E10</f>
         <v/>
       </c>
-      <c r="H10" s="18">
+      <c r="H10" s="19">
         <f>F10+G10</f>
         <v/>
       </c>
-      <c r="I10" s="18">
+      <c r="I10" s="19">
         <f>H10-BaselineSpend</f>
         <v/>
       </c>
-      <c r="J10" s="19">
+      <c r="J10" s="20">
         <f>IF(BaselineSpend=0,0,I10/BaselineSpend)</f>
         <v/>
       </c>
@@ -1295,209 +1314,209 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>APV $/drum  ↓   Split →</t>
         </is>
       </c>
-      <c r="B4" s="25" t="n">
+      <c r="B4" s="26" t="n">
         <v>0.1</v>
       </c>
-      <c r="C4" s="25" t="n">
+      <c r="C4" s="26" t="n">
         <v>0.2</v>
       </c>
-      <c r="D4" s="25" t="n">
+      <c r="D4" s="26" t="n">
         <v>0.25</v>
       </c>
-      <c r="E4" s="25" t="n">
+      <c r="E4" s="26" t="n">
         <v>0.33</v>
       </c>
-      <c r="F4" s="25" t="n">
+      <c r="F4" s="26" t="n">
         <v>0.5</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="n">
+      <c r="A5" s="13" t="n">
         <v>337.5</v>
       </c>
-      <c r="B5" s="18">
+      <c r="B5" s="19">
         <f>DrumsYr*(1-0.1)*SNPdrum + DrumsYr*0.1*$A5</f>
         <v/>
       </c>
-      <c r="C5" s="18">
+      <c r="C5" s="19">
         <f>DrumsYr*(1-0.2)*SNPdrum + DrumsYr*0.2*$A5</f>
         <v/>
       </c>
-      <c r="D5" s="18">
+      <c r="D5" s="19">
         <f>DrumsYr*(1-0.25)*SNPdrum + DrumsYr*0.25*$A5</f>
         <v/>
       </c>
-      <c r="E5" s="18">
+      <c r="E5" s="19">
         <f>DrumsYr*(1-0.33)*SNPdrum + DrumsYr*0.33*$A5</f>
         <v/>
       </c>
-      <c r="F5" s="18">
+      <c r="F5" s="19">
         <f>DrumsYr*(1-0.5)*SNPdrum + DrumsYr*0.5*$A5</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="n">
+      <c r="A6" s="13" t="n">
         <v>400</v>
       </c>
-      <c r="B6" s="18">
+      <c r="B6" s="19">
         <f>DrumsYr*(1-0.1)*SNPdrum + DrumsYr*0.1*$A6</f>
         <v/>
       </c>
-      <c r="C6" s="18">
+      <c r="C6" s="19">
         <f>DrumsYr*(1-0.2)*SNPdrum + DrumsYr*0.2*$A6</f>
         <v/>
       </c>
-      <c r="D6" s="18">
+      <c r="D6" s="19">
         <f>DrumsYr*(1-0.25)*SNPdrum + DrumsYr*0.25*$A6</f>
         <v/>
       </c>
-      <c r="E6" s="18">
+      <c r="E6" s="19">
         <f>DrumsYr*(1-0.33)*SNPdrum + DrumsYr*0.33*$A6</f>
         <v/>
       </c>
-      <c r="F6" s="18">
+      <c r="F6" s="19">
         <f>DrumsYr*(1-0.5)*SNPdrum + DrumsYr*0.5*$A6</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="n">
+      <c r="A7" s="13" t="n">
         <v>450</v>
       </c>
-      <c r="B7" s="18">
+      <c r="B7" s="19">
         <f>DrumsYr*(1-0.1)*SNPdrum + DrumsYr*0.1*$A7</f>
         <v/>
       </c>
-      <c r="C7" s="18">
+      <c r="C7" s="19">
         <f>DrumsYr*(1-0.2)*SNPdrum + DrumsYr*0.2*$A7</f>
         <v/>
       </c>
-      <c r="D7" s="18">
+      <c r="D7" s="19">
         <f>DrumsYr*(1-0.25)*SNPdrum + DrumsYr*0.25*$A7</f>
         <v/>
       </c>
-      <c r="E7" s="18">
+      <c r="E7" s="19">
         <f>DrumsYr*(1-0.33)*SNPdrum + DrumsYr*0.33*$A7</f>
         <v/>
       </c>
-      <c r="F7" s="18">
+      <c r="F7" s="19">
         <f>DrumsYr*(1-0.5)*SNPdrum + DrumsYr*0.5*$A7</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="n">
+      <c r="A8" s="13" t="n">
         <v>506.25</v>
       </c>
-      <c r="B8" s="18">
+      <c r="B8" s="19">
         <f>DrumsYr*(1-0.1)*SNPdrum + DrumsYr*0.1*$A8</f>
         <v/>
       </c>
-      <c r="C8" s="18">
+      <c r="C8" s="19">
         <f>DrumsYr*(1-0.2)*SNPdrum + DrumsYr*0.2*$A8</f>
         <v/>
       </c>
-      <c r="D8" s="18">
+      <c r="D8" s="19">
         <f>DrumsYr*(1-0.25)*SNPdrum + DrumsYr*0.25*$A8</f>
         <v/>
       </c>
-      <c r="E8" s="18">
+      <c r="E8" s="19">
         <f>DrumsYr*(1-0.33)*SNPdrum + DrumsYr*0.33*$A8</f>
         <v/>
       </c>
-      <c r="F8" s="18">
+      <c r="F8" s="19">
         <f>DrumsYr*(1-0.5)*SNPdrum + DrumsYr*0.5*$A8</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="n">
+      <c r="A9" s="13" t="n">
         <v>600</v>
       </c>
-      <c r="B9" s="18">
+      <c r="B9" s="19">
         <f>DrumsYr*(1-0.1)*SNPdrum + DrumsYr*0.1*$A9</f>
         <v/>
       </c>
-      <c r="C9" s="18">
+      <c r="C9" s="19">
         <f>DrumsYr*(1-0.2)*SNPdrum + DrumsYr*0.2*$A9</f>
         <v/>
       </c>
-      <c r="D9" s="18">
+      <c r="D9" s="19">
         <f>DrumsYr*(1-0.25)*SNPdrum + DrumsYr*0.25*$A9</f>
         <v/>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="19">
         <f>DrumsYr*(1-0.33)*SNPdrum + DrumsYr*0.33*$A9</f>
         <v/>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="19">
         <f>DrumsYr*(1-0.5)*SNPdrum + DrumsYr*0.5*$A9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="n">
+      <c r="A10" s="13" t="n">
         <v>675</v>
       </c>
-      <c r="B10" s="18">
+      <c r="B10" s="19">
         <f>DrumsYr*(1-0.1)*SNPdrum + DrumsYr*0.1*$A10</f>
         <v/>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="19">
         <f>DrumsYr*(1-0.2)*SNPdrum + DrumsYr*0.2*$A10</f>
         <v/>
       </c>
-      <c r="D10" s="18">
+      <c r="D10" s="19">
         <f>DrumsYr*(1-0.25)*SNPdrum + DrumsYr*0.25*$A10</f>
         <v/>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="19">
         <f>DrumsYr*(1-0.33)*SNPdrum + DrumsYr*0.33*$A10</f>
         <v/>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="19">
         <f>DrumsYr*(1-0.5)*SNPdrum + DrumsYr*0.5*$A10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="n">
+      <c r="A11" s="13" t="n">
         <v>750</v>
       </c>
-      <c r="B11" s="18">
+      <c r="B11" s="19">
         <f>DrumsYr*(1-0.1)*SNPdrum + DrumsYr*0.1*$A11</f>
         <v/>
       </c>
-      <c r="C11" s="18">
+      <c r="C11" s="19">
         <f>DrumsYr*(1-0.2)*SNPdrum + DrumsYr*0.2*$A11</f>
         <v/>
       </c>
-      <c r="D11" s="18">
+      <c r="D11" s="19">
         <f>DrumsYr*(1-0.25)*SNPdrum + DrumsYr*0.25*$A11</f>
         <v/>
       </c>
-      <c r="E11" s="18">
+      <c r="E11" s="19">
         <f>DrumsYr*(1-0.33)*SNPdrum + DrumsYr*0.33*$A11</f>
         <v/>
       </c>
-      <c r="F11" s="18">
+      <c r="F11" s="19">
         <f>DrumsYr*(1-0.5)*SNPdrum + DrumsYr*0.5*$A11</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="26" t="inlineStr">
+      <c r="A13" s="27" t="inlineStr">
         <is>
           <t>Baseline all-SNP for reference:</t>
         </is>
       </c>
-      <c r="C13" s="27">
+      <c r="C13" s="28">
         <f>BaselineSpend</f>
         <v/>
       </c>
@@ -1552,212 +1571,212 @@
       </c>
     </row>
     <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>SNP surcharge %</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>SNP $/drum</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>SNP annual (75%)</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="D4" s="16" t="inlineStr">
         <is>
           <t>APV annual (25%)</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>TOTAL annual</t>
         </is>
       </c>
-      <c r="F4" s="15" t="inlineStr">
+      <c r="F4" s="16" t="inlineStr">
         <is>
           <t>Δ vs all-SNP</t>
         </is>
       </c>
-      <c r="G4" s="15" t="inlineStr">
+      <c r="G4" s="16" t="inlineStr">
         <is>
           <t>Verdict</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="n">
+      <c r="A5" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="B5" s="18">
+      <c r="B5" s="19">
         <f>SNPdrum*(1+A5)</f>
         <v/>
       </c>
-      <c r="C5" s="18">
+      <c r="C5" s="19">
         <f>DrumsYr*(1-0.25)*B5</f>
         <v/>
       </c>
-      <c r="D5" s="18">
+      <c r="D5" s="19">
         <f>DrumsYr*0.25*APVlikely</f>
         <v/>
       </c>
-      <c r="E5" s="18">
+      <c r="E5" s="19">
         <f>C5+D5</f>
         <v/>
       </c>
-      <c r="F5" s="18">
+      <c r="F5" s="19">
         <f>E5-BaselineSpend</f>
         <v/>
       </c>
-      <c r="G5" s="28">
+      <c r="G5" s="29">
         <f>IF(F5&lt;=0,"Cheaper than baseline","Premium for redundancy: "&amp;TEXT(F5,"$#,##0"))</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="n">
+      <c r="A6" s="17" t="n">
         <v>0.05</v>
       </c>
-      <c r="B6" s="18">
+      <c r="B6" s="19">
         <f>SNPdrum*(1+A6)</f>
         <v/>
       </c>
-      <c r="C6" s="18">
+      <c r="C6" s="19">
         <f>DrumsYr*(1-0.25)*B6</f>
         <v/>
       </c>
-      <c r="D6" s="18">
+      <c r="D6" s="19">
         <f>DrumsYr*0.25*APVlikely</f>
         <v/>
       </c>
-      <c r="E6" s="18">
+      <c r="E6" s="19">
         <f>C6+D6</f>
         <v/>
       </c>
-      <c r="F6" s="18">
+      <c r="F6" s="19">
         <f>E6-BaselineSpend</f>
         <v/>
       </c>
-      <c r="G6" s="28">
+      <c r="G6" s="29">
         <f>IF(F6&lt;=0,"Cheaper than baseline","Premium for redundancy: "&amp;TEXT(F6,"$#,##0"))</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="n">
+      <c r="A7" s="17" t="n">
         <v>0.1</v>
       </c>
-      <c r="B7" s="18">
+      <c r="B7" s="19">
         <f>SNPdrum*(1+A7)</f>
         <v/>
       </c>
-      <c r="C7" s="18">
+      <c r="C7" s="19">
         <f>DrumsYr*(1-0.25)*B7</f>
         <v/>
       </c>
-      <c r="D7" s="18">
+      <c r="D7" s="19">
         <f>DrumsYr*0.25*APVlikely</f>
         <v/>
       </c>
-      <c r="E7" s="18">
+      <c r="E7" s="19">
         <f>C7+D7</f>
         <v/>
       </c>
-      <c r="F7" s="18">
+      <c r="F7" s="19">
         <f>E7-BaselineSpend</f>
         <v/>
       </c>
-      <c r="G7" s="28">
+      <c r="G7" s="29">
         <f>IF(F7&lt;=0,"Cheaper than baseline","Premium for redundancy: "&amp;TEXT(F7,"$#,##0"))</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="n">
+      <c r="A8" s="17" t="n">
         <v>0.15</v>
       </c>
-      <c r="B8" s="18">
+      <c r="B8" s="19">
         <f>SNPdrum*(1+A8)</f>
         <v/>
       </c>
-      <c r="C8" s="18">
+      <c r="C8" s="19">
         <f>DrumsYr*(1-0.25)*B8</f>
         <v/>
       </c>
-      <c r="D8" s="18">
+      <c r="D8" s="19">
         <f>DrumsYr*0.25*APVlikely</f>
         <v/>
       </c>
-      <c r="E8" s="18">
+      <c r="E8" s="19">
         <f>C8+D8</f>
         <v/>
       </c>
-      <c r="F8" s="18">
+      <c r="F8" s="19">
         <f>E8-BaselineSpend</f>
         <v/>
       </c>
-      <c r="G8" s="28">
+      <c r="G8" s="29">
         <f>IF(F8&lt;=0,"Cheaper than baseline","Premium for redundancy: "&amp;TEXT(F8,"$#,##0"))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="n">
+      <c r="A9" s="17" t="n">
         <v>0.2</v>
       </c>
-      <c r="B9" s="18">
+      <c r="B9" s="19">
         <f>SNPdrum*(1+A9)</f>
         <v/>
       </c>
-      <c r="C9" s="18">
+      <c r="C9" s="19">
         <f>DrumsYr*(1-0.25)*B9</f>
         <v/>
       </c>
-      <c r="D9" s="18">
+      <c r="D9" s="19">
         <f>DrumsYr*0.25*APVlikely</f>
         <v/>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="19">
         <f>C9+D9</f>
         <v/>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="19">
         <f>E9-BaselineSpend</f>
         <v/>
       </c>
-      <c r="G9" s="28">
+      <c r="G9" s="29">
         <f>IF(F9&lt;=0,"Cheaper than baseline","Premium for redundancy: "&amp;TEXT(F9,"$#,##0"))</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="n">
+      <c r="A10" s="17" t="n">
         <v>0.25</v>
       </c>
-      <c r="B10" s="18">
+      <c r="B10" s="19">
         <f>SNPdrum*(1+A10)</f>
         <v/>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="19">
         <f>DrumsYr*(1-0.25)*B10</f>
         <v/>
       </c>
-      <c r="D10" s="18">
+      <c r="D10" s="19">
         <f>DrumsYr*0.25*APVlikely</f>
         <v/>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="19">
         <f>C10+D10</f>
         <v/>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="19">
         <f>E10-BaselineSpend</f>
         <v/>
       </c>
-      <c r="G10" s="28">
+      <c r="G10" s="29">
         <f>IF(F10&lt;=0,"Cheaper than baseline","Premium for redundancy: "&amp;TEXT(F10,"$#,##0"))</f>
         <v/>
       </c>
@@ -1808,299 +1827,299 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Will a tiny (~$5k-$35k/yr), intermittent single-drum account be attractive? Sizes are rough public estimates.</t>
+          <t>Total account ~$50k/yr (1,300 lb/wk); a 20-25% 2nd-source slice = ~$12-19k/yr. Will that be attractive to each? Sizes are rough public estimates.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>Supplier</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="D4" s="16" t="inlineStr">
         <is>
           <t>Est. size</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>Min batch</t>
         </is>
       </c>
-      <c r="F4" s="15" t="inlineStr">
+      <c r="F4" s="16" t="inlineStr">
         <is>
           <t>Meets single-drum order?</t>
         </is>
       </c>
-      <c r="G4" s="15" t="inlineStr">
+      <c r="G4" s="16" t="inlineStr">
         <is>
           <t>Small-acct fit</t>
         </is>
       </c>
-      <c r="H4" s="15" t="inlineStr">
+      <c r="H4" s="16" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>SNP (incumbent)</t>
         </is>
       </c>
-      <c r="B5" s="28" t="inlineStr">
+      <c r="B5" s="29" t="inlineStr">
         <is>
           <t>Specialty chem / PVA maker</t>
         </is>
       </c>
-      <c r="C5" s="28" t="inlineStr">
+      <c r="C5" s="29" t="inlineStr">
         <is>
           <t>Durham, NC</t>
         </is>
       </c>
-      <c r="D5" s="28" t="inlineStr">
+      <c r="D5" s="29" t="inlineStr">
         <is>
           <t>~$4M, ~small</t>
         </is>
       </c>
-      <c r="E5" s="28" t="inlineStr">
+      <c r="E5" s="29" t="inlineStr">
         <is>
           <t>n/a (incumbent)</t>
         </is>
       </c>
-      <c r="F5" s="28" t="inlineStr">
+      <c r="F5" s="29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G5" s="29" t="inlineStr">
+      <c r="G5" s="30" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="H5" s="28" t="inlineStr">
+      <c r="H5" s="29" t="inlineStr">
         <is>
           <t>PVA + alginates are core products; already your supplier. Best natural fit; main risk is small-vendor continuity.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="28" t="inlineStr">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>APV Engineered Coatings</t>
         </is>
       </c>
-      <c r="B6" s="28" t="inlineStr">
+      <c r="B6" s="29" t="inlineStr">
         <is>
           <t>Coatings maker + contract mfg</t>
         </is>
       </c>
-      <c r="C6" s="28" t="inlineStr">
+      <c r="C6" s="29" t="inlineStr">
         <is>
           <t>Akron, OH</t>
         </is>
       </c>
-      <c r="D6" s="28" t="inlineStr">
+      <c r="D6" s="29" t="inlineStr">
         <is>
           <t>~$28M, ~50-200 emp</t>
         </is>
       </c>
-      <c r="E6" s="28" t="inlineStr">
+      <c r="E6" s="29" t="inlineStr">
         <is>
           <t>100 gal (~2 drums)</t>
         </is>
       </c>
-      <c r="F6" s="28" t="inlineStr">
+      <c r="F6" s="29" t="inlineStr">
         <is>
           <t>Below min for 1 drum; order 2-drum runs</t>
         </is>
       </c>
-      <c r="G6" s="30" t="inlineStr">
+      <c r="G6" s="31" t="inlineStr">
         <is>
           <t>Neutral / verify</t>
         </is>
       </c>
-      <c r="H6" s="28" t="inlineStr">
+      <c r="H6" s="29" t="inlineStr">
         <is>
           <t>Confirmed 95C heating (gate cleared). 100-gal min batch + own product lines -&gt; may price single drums at a premium. STRONGEST new lead on capability.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="28" t="inlineStr">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t>ArroChem</t>
         </is>
       </c>
-      <c r="B7" s="28" t="inlineStr">
+      <c r="B7" s="29" t="inlineStr">
         <is>
           <t>Family toll blender</t>
         </is>
       </c>
-      <c r="C7" s="28" t="inlineStr">
+      <c r="C7" s="29" t="inlineStr">
         <is>
           <t>Mt Holly, NC</t>
         </is>
       </c>
-      <c r="D7" s="28" t="inlineStr">
+      <c r="D7" s="29" t="inlineStr">
         <is>
           <t>family-owned, 1 site</t>
         </is>
       </c>
-      <c r="E7" s="28" t="inlineStr">
+      <c r="E7" s="29" t="inlineStr">
         <is>
           <t>55 gal (1 drum)</t>
         </is>
       </c>
-      <c r="F7" s="28" t="inlineStr">
+      <c r="F7" s="29" t="inlineStr">
         <is>
           <t>Yes - exact match</t>
         </is>
       </c>
-      <c r="G7" s="29" t="inlineStr">
+      <c r="G7" s="30" t="inlineStr">
         <is>
           <t>Good (capability TBD)</t>
         </is>
       </c>
-      <c r="H7" s="28" t="inlineStr">
+      <c r="H7" s="29" t="inlineStr">
         <is>
           <t>Advertised 55-5,000 gal batches = single drum is their floor. BUT failed trial: could not reach 95C. Re-confirm heating before relying on them.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="28" t="inlineStr">
+      <c r="A8" s="29" t="inlineStr">
         <is>
           <t>Carolina Solvents</t>
         </is>
       </c>
-      <c r="B8" s="28" t="inlineStr">
+      <c r="B8" s="29" t="inlineStr">
         <is>
           <t>Small solvent/coating shop</t>
         </is>
       </c>
-      <c r="C8" s="28" t="inlineStr">
+      <c r="C8" s="29" t="inlineStr">
         <is>
           <t>Hickory, NC</t>
         </is>
       </c>
-      <c r="D8" s="28" t="inlineStr">
+      <c r="D8" s="29" t="inlineStr">
         <is>
           <t>&lt;$5M, &lt;25 emp</t>
         </is>
       </c>
-      <c r="E8" s="28" t="inlineStr">
+      <c r="E8" s="29" t="inlineStr">
         <is>
           <t>unknown (small)</t>
         </is>
       </c>
-      <c r="F8" s="28" t="inlineStr">
+      <c r="F8" s="29" t="inlineStr">
         <is>
           <t>Likely yes</t>
         </is>
       </c>
-      <c r="G8" s="29" t="inlineStr">
+      <c r="G8" s="30" t="inlineStr">
         <is>
           <t>Good / verify process</t>
         </is>
       </c>
-      <c r="H8" s="28" t="inlineStr">
+      <c r="H8" s="29" t="inlineStr">
         <is>
           <t>Smallest -&gt; would value the account. Solvent/ambient focus; CONFIRM heated aqueous 95C capability. Not yet contacted.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="28" t="inlineStr">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>Piedmont Chemical</t>
         </is>
       </c>
-      <c r="B9" s="28" t="inlineStr">
+      <c r="B9" s="29" t="inlineStr">
         <is>
           <t>Custom synthesis/polymer</t>
         </is>
       </c>
-      <c r="C9" s="28" t="inlineStr">
+      <c r="C9" s="29" t="inlineStr">
         <is>
           <t>High Point, NC</t>
         </is>
       </c>
-      <c r="D9" s="28" t="inlineStr">
+      <c r="D9" s="29" t="inlineStr">
         <is>
           <t>~$35M, ~64-180 emp</t>
         </is>
       </c>
-      <c r="E9" s="28" t="inlineStr">
+      <c r="E9" s="29" t="inlineStr">
         <is>
           <t>unknown (larger)</t>
         </is>
       </c>
-      <c r="F9" s="28" t="inlineStr">
+      <c r="F9" s="29" t="inlineStr">
         <is>
           <t>Probably below their sweet spot</t>
         </is>
       </c>
-      <c r="G9" s="30" t="inlineStr">
+      <c r="G9" s="31" t="inlineStr">
         <is>
           <t>Caution / lean too big</t>
         </is>
       </c>
-      <c r="H9" s="28" t="inlineStr">
+      <c r="H9" s="29" t="inlineStr">
         <is>
           <t>Synthesis orientation wants bigger campaigns; a single-drum blend likely under-prioritized or premium-priced.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="28" t="inlineStr">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>ILC Dover</t>
         </is>
       </c>
-      <c r="B10" s="28" t="inlineStr">
+      <c r="B10" s="29" t="inlineStr">
         <is>
           <t>Pharma/aerospace (Ingersoll Rand)</t>
         </is>
       </c>
-      <c r="C10" s="28" t="inlineStr">
+      <c r="C10" s="29" t="inlineStr">
         <is>
           <t>Frederica, DE</t>
         </is>
       </c>
-      <c r="D10" s="28" t="inlineStr">
+      <c r="D10" s="29" t="inlineStr">
         <is>
           <t>$80M-$450M, ~2,100 emp</t>
         </is>
       </c>
-      <c r="E10" s="28" t="inlineStr">
+      <c r="E10" s="29" t="inlineStr">
         <is>
           <t>n/a - equipment/services</t>
         </is>
       </c>
-      <c r="F10" s="28" t="inlineStr">
+      <c r="F10" s="29" t="inlineStr">
         <is>
           <t>No - wrong category</t>
         </is>
       </c>
-      <c r="G10" s="31" t="inlineStr">
+      <c r="G10" s="32" t="inlineStr">
         <is>
           <t>Too big / wrong type</t>
         </is>
       </c>
-      <c r="H10" s="28" t="inlineStr">
+      <c r="H10" s="29" t="inlineStr">
         <is>
           <t>Could NOT reach 95C and is an equipment/containment firm, not a drum toll blender. Recommend deprioritize/close out.</t>
         </is>
@@ -2121,294 +2140,294 @@
       <c r="H12" s="3" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="28" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>Brenntag</t>
         </is>
       </c>
-      <c r="B13" s="28" t="inlineStr">
+      <c r="B13" s="29" t="inlineStr">
         <is>
           <t>World's largest chem distributor</t>
         </is>
       </c>
-      <c r="C13" s="28" t="inlineStr">
+      <c r="C13" s="29" t="inlineStr">
         <is>
           <t>Essen, DE / US-wide</t>
         </is>
       </c>
-      <c r="D13" s="28" t="inlineStr">
+      <c r="D13" s="29" t="inlineStr">
         <is>
           <t>~EUR15B, ~17k emp</t>
         </is>
       </c>
-      <c r="E13" s="28" t="inlineStr">
+      <c r="E13" s="29" t="inlineStr">
         <is>
           <t>single drums (core)</t>
         </is>
       </c>
-      <c r="F13" s="28" t="inlineStr">
+      <c r="F13" s="29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G13" s="30" t="inlineStr">
+      <c r="G13" s="31" t="inlineStr">
         <is>
           <t>Neutral (serve, no VIP)</t>
         </is>
       </c>
-      <c r="H13" s="28" t="inlineStr">
+      <c r="H13" s="29" t="inlineStr">
         <is>
           <t>Already lists Sekisui Selvol PVA -&gt; easiest source of genuine resin in drums. You'll be a small/transactional account; possible small-order premium.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="28" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>Tilley Distribution</t>
         </is>
       </c>
-      <c r="B14" s="28" t="inlineStr">
+      <c r="B14" s="29" t="inlineStr">
         <is>
           <t>Regional specialty distributor (PE-backed)</t>
         </is>
       </c>
-      <c r="C14" s="28" t="inlineStr">
+      <c r="C14" s="29" t="inlineStr">
         <is>
           <t>Baltimore, MD</t>
         </is>
       </c>
-      <c r="D14" s="28" t="inlineStr">
+      <c r="D14" s="29" t="inlineStr">
         <is>
           <t>~$40M, ~120-180 emp</t>
         </is>
       </c>
-      <c r="E14" s="28" t="inlineStr">
+      <c r="E14" s="29" t="inlineStr">
         <is>
           <t>drums/small lots</t>
         </is>
       </c>
-      <c r="F14" s="28" t="inlineStr">
+      <c r="F14" s="29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G14" s="29" t="inlineStr">
+      <c r="G14" s="30" t="inlineStr">
         <is>
           <t>Good (best relationship fit)</t>
         </is>
       </c>
-      <c r="H14" s="28" t="inlineStr">
+      <c r="H14" s="29" t="inlineStr">
         <is>
           <t>$25k account is meaningful to them; relationship-oriented. OPEN: confirm they actually source a PVA brand. Was already flagged as slow/maybe can't meet.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="inlineStr">
+      <c r="A15" s="29" t="inlineStr">
         <is>
           <t>Palmer Holland</t>
         </is>
       </c>
-      <c r="B15" s="28" t="inlineStr">
+      <c r="B15" s="29" t="inlineStr">
         <is>
           <t>Mid-size NA distributor (ESOP)</t>
         </is>
       </c>
-      <c r="C15" s="28" t="inlineStr">
+      <c r="C15" s="29" t="inlineStr">
         <is>
           <t>Westlake, OH</t>
         </is>
       </c>
-      <c r="D15" s="28" t="inlineStr">
+      <c r="D15" s="29" t="inlineStr">
         <is>
           <t>~250 emp, national</t>
         </is>
       </c>
-      <c r="E15" s="28" t="inlineStr">
+      <c r="E15" s="29" t="inlineStr">
         <is>
           <t>drums/specialty lots</t>
         </is>
       </c>
-      <c r="F15" s="28" t="inlineStr">
+      <c r="F15" s="29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G15" s="29" t="inlineStr">
+      <c r="G15" s="30" t="inlineStr">
         <is>
           <t>Good-Neutral</t>
         </is>
       </c>
-      <c r="H15" s="28" t="inlineStr">
+      <c r="H15" s="29" t="inlineStr">
         <is>
           <t>Employee-owned, relationship-driven, workable size. OPEN: confirm they carry a PVA principal (unverified).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="28" t="inlineStr">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>Barentz</t>
         </is>
       </c>
-      <c r="B16" s="28" t="inlineStr">
+      <c r="B16" s="29" t="inlineStr">
         <is>
           <t>Large global specialty distributor</t>
         </is>
       </c>
-      <c r="C16" s="28" t="inlineStr">
+      <c r="C16" s="29" t="inlineStr">
         <is>
           <t>Hoofddorp, NL / NA</t>
         </is>
       </c>
-      <c r="D16" s="28" t="inlineStr">
+      <c r="D16" s="29" t="inlineStr">
         <is>
           <t>~EUR2.4B, ~2,700 emp</t>
         </is>
       </c>
-      <c r="E16" s="28" t="inlineStr">
+      <c r="E16" s="29" t="inlineStr">
         <is>
           <t>drums (focus skews large)</t>
         </is>
       </c>
-      <c r="F16" s="28" t="inlineStr">
+      <c r="F16" s="29" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G16" s="31" t="inlineStr">
+      <c r="G16" s="32" t="inlineStr">
         <is>
           <t>Likely too big to prioritize</t>
         </is>
       </c>
-      <c r="H16" s="28" t="inlineStr">
+      <c r="H16" s="29" t="inlineStr">
         <is>
           <t>Lists PVA and can serve, but a tiny industrial-drum account isn't their priority segment.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="28" t="inlineStr">
+      <c r="A17" s="29" t="inlineStr">
         <is>
           <t>Sekisui Specialty Chem</t>
         </is>
       </c>
-      <c r="B17" s="28" t="inlineStr">
+      <c r="B17" s="29" t="inlineStr">
         <is>
           <t>PVA PRODUCER (Selvol)</t>
         </is>
       </c>
-      <c r="C17" s="28" t="inlineStr">
+      <c r="C17" s="29" t="inlineStr">
         <is>
           <t>Dallas, TX</t>
         </is>
       </c>
-      <c r="D17" s="28" t="inlineStr">
+      <c r="D17" s="29" t="inlineStr">
         <is>
           <t>~$186M US, ~260-400 emp</t>
         </is>
       </c>
-      <c r="E17" s="28" t="inlineStr">
+      <c r="E17" s="29" t="inlineStr">
         <is>
           <t>bulk; NOT direct</t>
         </is>
       </c>
-      <c r="F17" s="28" t="inlineStr">
+      <c r="F17" s="29" t="inlineStr">
         <is>
           <t>No (via distributor)</t>
         </is>
       </c>
-      <c r="G17" s="31" t="inlineStr">
+      <c r="G17" s="32" t="inlineStr">
         <is>
           <t>Too small to buy direct</t>
         </is>
       </c>
-      <c r="H17" s="28" t="inlineStr">
+      <c r="H17" s="29" t="inlineStr">
         <is>
           <t>It IS Selvol (your reference resin). Won't sell factory-direct at your volume -&gt; routes you to Brenntag etc.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="28" t="inlineStr">
+      <c r="A18" s="29" t="inlineStr">
         <is>
           <t>Kuraray</t>
         </is>
       </c>
-      <c r="B18" s="28" t="inlineStr">
+      <c r="B18" s="29" t="inlineStr">
         <is>
           <t>World's largest PVA PRODUCER</t>
         </is>
       </c>
-      <c r="C18" s="28" t="inlineStr">
+      <c r="C18" s="29" t="inlineStr">
         <is>
           <t>Tokyo / Houston TX</t>
         </is>
       </c>
-      <c r="D18" s="28" t="inlineStr">
+      <c r="D18" s="29" t="inlineStr">
         <is>
           <t>~$5.4B, ~12k emp</t>
         </is>
       </c>
-      <c r="E18" s="28" t="inlineStr">
+      <c r="E18" s="29" t="inlineStr">
         <is>
           <t>bulk; NOT direct</t>
         </is>
       </c>
-      <c r="F18" s="28" t="inlineStr">
+      <c r="F18" s="29" t="inlineStr">
         <is>
           <t>No (via distributor)</t>
         </is>
       </c>
-      <c r="G18" s="31" t="inlineStr">
+      <c r="G18" s="32" t="inlineStr">
         <is>
           <t>Too small to buy direct</t>
         </is>
       </c>
-      <c r="H18" s="28" t="inlineStr">
+      <c r="H18" s="29" t="inlineStr">
         <is>
           <t>Poval/Elvanol brand owner. Buy via named distributors: dar-tech (Buffalo NY, closest East Coast) or Associated Agencies.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="28" t="inlineStr">
+      <c r="A19" s="29" t="inlineStr">
         <is>
           <t>Aldon Corp</t>
         </is>
       </c>
-      <c r="B19" s="28" t="inlineStr">
+      <c r="B19" s="29" t="inlineStr">
         <is>
           <t>Lab/education chem + contract blender</t>
         </is>
       </c>
-      <c r="C19" s="28" t="inlineStr">
+      <c r="C19" s="29" t="inlineStr">
         <is>
           <t>Avon, NY</t>
         </is>
       </c>
-      <c r="D19" s="28" t="inlineStr">
+      <c r="D19" s="29" t="inlineStr">
         <is>
           <t>small, private</t>
         </is>
       </c>
-      <c r="E19" s="28" t="inlineStr">
+      <c r="E19" s="29" t="inlineStr">
         <is>
           <t>lab bottles, not drums</t>
         </is>
       </c>
-      <c r="F19" s="28" t="inlineStr">
+      <c r="F19" s="29" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G19" s="31" t="inlineStr">
+      <c r="G19" s="32" t="inlineStr">
         <is>
           <t>Poor / wrong type</t>
         </is>
       </c>
-      <c r="H19" s="28" t="inlineStr">
+      <c r="H19" s="29" t="inlineStr">
         <is>
           <t>Education &amp; private-label LAB-grade PVA solutions only. Not an industrial drum-resin source. Close out.</t>
         </is>

</xml_diff>

<commit_message>
Update supplier roster: new US candidates + volume feasibility
- Regroup suppliers by status: active shortlist / advisor / dropped / eliminated
- Add CJB Applied Technologies, Columbus Chemical (CCI), CORECHEM, Northstar,
  plus dropped (Goulston, 3V Sigma, Royal, Columbia) and Sekisui as advisor
- Correct APV min batch to ~5 gal (was 100); upgrade Piedmont to GOOD fit
- Add volume-feasibility read vs ~1 drum/wk slice under 18-day shelf life
  (flag CORECHEM 250-gal and Royal 220-gal MOQ as shelf-life overshoot)
- Mark ArroChem eliminated (85 C ceiling)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkE2ZRYs3PLyj8XHTsU3i4
</commit_message>
<xml_diff>
--- a/PVA_Second_Source_Pricing_Model.xlsx
+++ b/PVA_Second_Source_Pricing_Model.xlsx
@@ -9,9 +9,9 @@
   <sheets>
     <sheet name="Inputs &amp; Assumptions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Split Scenarios" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="APV Price Sensitivity" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Price Sensitivity" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="SNP Re-pricing Risk" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Supplier Capacity" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Supplier Roster" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="DrumGal">'Inputs &amp; Assumptions'!$C$6</definedName>
@@ -24,7 +24,7 @@
     <definedName name="DrumsYr">'Inputs &amp; Assumptions'!$C$13</definedName>
     <definedName name="GalYr">'Inputs &amp; Assumptions'!$C$14</definedName>
     <definedName name="BaselineSpend">'Inputs &amp; Assumptions'!$C$15</definedName>
-    <definedName name="APVminGal">'Inputs &amp; Assumptions'!$C$18</definedName>
+    <definedName name="MinBatch">'Inputs &amp; Assumptions'!$C$18</definedName>
     <definedName name="APVlow">'Inputs &amp; Assumptions'!$C$19</definedName>
     <definedName name="APVlikely">'Inputs &amp; Assumptions'!$C$20</definedName>
     <definedName name="APVhigh">'Inputs &amp; Assumptions'!$C$21</definedName>
@@ -42,7 +42,7 @@
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -81,8 +81,12 @@
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -116,12 +120,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00404040"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00A9D08E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
     <fill>
@@ -156,7 +175,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -235,14 +254,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -609,14 +637,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E32"/>
+  <dimension ref="B2:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -629,7 +657,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Working model. Edit only the YELLOW cells; green cells are calculated. Built 2026-06-26.</t>
+          <t>Working model. Edit only the YELLOW cells; green cells are calculated. Updated 2026-06-26.</t>
         </is>
       </c>
     </row>
@@ -640,7 +668,7 @@
         </is>
       </c>
       <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
@@ -693,7 +721,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Confirmed by Oscar 2026-06-26: ~1,300 lb finished liquid/wk. This is how SNP bills (per lb). Supersedes the old 55 vs 220 gal estimates.</t>
+          <t>Confirmed by Oscar 2026-06-26: ~1,300 lb finished liquid/wk. This is how SNP bills (per lb).</t>
         </is>
       </c>
     </row>
@@ -783,7 +811,7 @@
     <row r="17">
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>2) APV / SECOND-SOURCE PRICE ASSUMPTIONS (placeholders until real quote)</t>
+          <t>2) SECOND-SOURCE PRICE ASSUMPTIONS (placeholders until real quote)</t>
         </is>
       </c>
       <c r="C17" s="3" t="n"/>
@@ -792,22 +820,22 @@
     <row r="18">
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>APV minimum batch (gallons)</t>
+          <t>Min batch of best small-batch candidates (gal)</t>
         </is>
       </c>
       <c r="C18" s="5" t="n">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>APV Engineered Coatings advertises 100-8,700 gal batches. A single 55-gal drum is BELOW min -&gt; order in 2-drum (110 gal) runs to be efficient.</t>
+          <t>Corrected 2026-06-26: APV / Piedmont / Columbus all run from ~5 gal. A single drum (55 gal) is easily within a batch.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>APV price/drum - LOW (best case)</t>
+          <t>2nd-source price/drum - LOW (best case)</t>
         </is>
       </c>
       <c r="C19" s="13">
@@ -816,14 +844,14 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Parity with SNP. Unlikely at low volume; optimistic floor.</t>
+          <t>Parity with SNP. Optimistic floor.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>APV price/drum - LIKELY</t>
+          <t>2nd-source price/drum - LIKELY</t>
         </is>
       </c>
       <c r="C20" s="13">
@@ -832,14 +860,14 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>+50% small-batch premium. ADJUST when APV quotes.</t>
+          <t>+50% small-batch premium. ADJUST when a real quote lands.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>APV price/drum - HIGH (single-drum penalty)</t>
+          <t>2nd-source price/drum - HIGH</t>
         </is>
       </c>
       <c r="C21" s="13">
@@ -848,7 +876,7 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>+100%: pays for ~100-gal min batch to make one drum.</t>
+          <t>+100% worst case.</t>
         </is>
       </c>
     </row>
@@ -872,7 +900,7 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Set e.g. 10% to test: does SNP raise the rate on remaining drums once they lose the full account? Used in scenarios.</t>
+          <t>Set e.g. 10% to test whether SNP raises the rate on remaining drums. Used in scenarios.</t>
         </is>
       </c>
     </row>
@@ -886,42 +914,49 @@
     <row r="27">
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Tab 'Split Scenarios': compare giving APV 0/10/20/25/33/50% of volume at the LIKELY price.</t>
+          <t xml:space="preserve">  - 'Split Scenarios': compare giving the 2nd source 0/10/20/25/33/50% of volume at the LIKELY price.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Tab 'APV Price Sensitivity': how total cost moves with APV's real quote x the split.</t>
+          <t xml:space="preserve">  - 'Price Sensitivity': how total cost moves with the real per-drum quote x the split.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Tab 'SNP Re-pricing Risk': the breakeven - how big an SNP surcharge erases the value of a 2nd source.</t>
+          <t xml:space="preserve">  - 'SNP Re-pricing Risk': breakeven - how big an SNP surcharge erases the value of a 2nd source.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Tab 'Supplier Capacity': who is big/small and whether a single-drum account fits them.</t>
+          <t xml:space="preserve">  - 'Supplier Roster': US candidates grouped by status + volume feasibility for a ~1 drum/wk slice.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>DECIDED: fixed split ~20-25% to APV (~quote per drum, recurring rotation). Highlighted in Split Scenarios.</t>
+          <t>DECIDED: fixed split ~20-25% to the 2nd source (~30-38 drums/yr), quoted per drum as a recurring rotation.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>REMEMBER: real viscosity target is still pending from SNP CoA history - APV cannot finalize a firm quote without it.</t>
+          <t>GATING for any firm quote: viscosity target still pending from SNP CoA history.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>SECOND-SOURCE SLICE (~1 drum/wk) + 18-day shelf life =&gt; prefer suppliers with a SMALL min batch so you don't make more than ~2 drums you can use in time.</t>
         </is>
       </c>
     </row>
@@ -939,13 +974,13 @@
   <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
@@ -954,26 +989,26 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Volume-Split Scenarios  (APV priced at LIKELY; SNP includes any surcharge from Inputs)</t>
+          <t>Volume-Split Scenarios  (2nd source priced at LIKELY; SNP includes any surcharge from Inputs)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Each row = a different share of total annual drums sent to APV (2nd source). SNP keeps the rest.</t>
+          <t>Each row = a different share of total annual drums sent to the 2nd source. SNP keeps the rest.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
-          <t>Split % to APV</t>
+          <t>Split % to 2nd src</t>
         </is>
       </c>
       <c r="B4" s="16" t="inlineStr">
         <is>
-          <t>APV drums/yr</t>
+          <t>2nd-src drums/yr</t>
         </is>
       </c>
       <c r="C4" s="16" t="inlineStr">
@@ -989,7 +1024,7 @@
       </c>
       <c r="E4" s="16" t="inlineStr">
         <is>
-          <t>APV $/drum
+          <t>2nd-src $/drum
 (Likely)</t>
         </is>
       </c>
@@ -1000,7 +1035,7 @@
       </c>
       <c r="G4" s="16" t="inlineStr">
         <is>
-          <t>APV annual $</t>
+          <t>2nd-src annual $</t>
         </is>
       </c>
       <c r="H4" s="16" t="inlineStr">
@@ -1268,7 +1303,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Highlighted rows (20% / 25%) = the decided fixed-split range. 'Δ vs all-SNP' is the annual cost of redundancy.</t>
+          <t>Highlighted rows (20% / 25%) = decided fixed-split range. 'Δ vs all-SNP' = annual cost of redundancy.</t>
         </is>
       </c>
     </row>
@@ -1302,21 +1337,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>APV Price Sensitivity — TOTAL annual cost ($)</t>
+          <t>2nd-Source Price Sensitivity — TOTAL annual cost ($)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rows = APV's actual price per drum (fill in once they quote). Cols = % of volume to APV. SNP at base (no surcharge here).</t>
+          <t>Rows = the 2nd source's actual price per drum (fill in once they quote). Cols = % of volume to them. SNP at base.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="25" t="inlineStr">
         <is>
-          <t>APV $/drum  ↓   Split →</t>
+          <t>$/drum  ↓   Split →</t>
         </is>
       </c>
       <c r="B4" s="26" t="n">
@@ -1513,7 +1548,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>Baseline all-SNP for reference:</t>
+          <t>Baseline all-SNP:</t>
         </is>
       </c>
       <c r="C13" s="28">
@@ -1524,7 +1559,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Yellow column = type APV's real per-drum quote here to read total cost across splits.</t>
+          <t>Yellow column = type the real per-drum quote here to read total cost across splits.</t>
         </is>
       </c>
     </row>
@@ -1550,7 +1585,7 @@
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
@@ -1566,7 +1601,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Scenario: 25% to APV at LIKELY price; SNP applies a surcharge on its remaining 75%. Shows when a 2nd source turns net-negative.</t>
+          <t>Scenario: 25% to 2nd source at LIKELY price; SNP applies a surcharge on its remaining 75%.</t>
         </is>
       </c>
     </row>
@@ -1588,7 +1623,7 @@
       </c>
       <c r="D4" s="16" t="inlineStr">
         <is>
-          <t>APV annual (25%)</t>
+          <t>2nd-src annual (25%)</t>
         </is>
       </c>
       <c r="E4" s="16" t="inlineStr">
@@ -1632,7 +1667,7 @@
         <v/>
       </c>
       <c r="G5" s="29">
-        <f>IF(F5&lt;=0,"Cheaper than baseline","Premium for redundancy: "&amp;TEXT(F5,"$#,##0"))</f>
+        <f>IF(F5&lt;=0,"Cheaper than baseline","Redundancy premium: "&amp;TEXT(F5,"$#,##0"))</f>
         <v/>
       </c>
     </row>
@@ -1661,7 +1696,7 @@
         <v/>
       </c>
       <c r="G6" s="29">
-        <f>IF(F6&lt;=0,"Cheaper than baseline","Premium for redundancy: "&amp;TEXT(F6,"$#,##0"))</f>
+        <f>IF(F6&lt;=0,"Cheaper than baseline","Redundancy premium: "&amp;TEXT(F6,"$#,##0"))</f>
         <v/>
       </c>
     </row>
@@ -1690,7 +1725,7 @@
         <v/>
       </c>
       <c r="G7" s="29">
-        <f>IF(F7&lt;=0,"Cheaper than baseline","Premium for redundancy: "&amp;TEXT(F7,"$#,##0"))</f>
+        <f>IF(F7&lt;=0,"Cheaper than baseline","Redundancy premium: "&amp;TEXT(F7,"$#,##0"))</f>
         <v/>
       </c>
     </row>
@@ -1719,7 +1754,7 @@
         <v/>
       </c>
       <c r="G8" s="29">
-        <f>IF(F8&lt;=0,"Cheaper than baseline","Premium for redundancy: "&amp;TEXT(F8,"$#,##0"))</f>
+        <f>IF(F8&lt;=0,"Cheaper than baseline","Redundancy premium: "&amp;TEXT(F8,"$#,##0"))</f>
         <v/>
       </c>
     </row>
@@ -1748,7 +1783,7 @@
         <v/>
       </c>
       <c r="G9" s="29">
-        <f>IF(F9&lt;=0,"Cheaper than baseline","Premium for redundancy: "&amp;TEXT(F9,"$#,##0"))</f>
+        <f>IF(F9&lt;=0,"Cheaper than baseline","Redundancy premium: "&amp;TEXT(F9,"$#,##0"))</f>
         <v/>
       </c>
     </row>
@@ -1777,14 +1812,14 @@
         <v/>
       </c>
       <c r="G10" s="29">
-        <f>IF(F10&lt;=0,"Cheaper than baseline","Premium for redundancy: "&amp;TEXT(F10,"$#,##0"))</f>
+        <f>IF(F10&lt;=0,"Cheaper than baseline","Redundancy premium: "&amp;TEXT(F10,"$#,##0"))</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Read: the redundancy 'premium' = APV's higher price + any SNP surcharge. This quantifies the insurance cost of a 2nd source.</t>
+          <t>The redundancy 'premium' = the 2nd source's higher price + any SNP surcharge = the insurance cost of dual-sourcing.</t>
         </is>
       </c>
     </row>
@@ -1804,30 +1839,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Supplier Size &amp; Small-Account Fit</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+          <t>Supplier Roster &amp; Volume Feasibility  (US-only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total account ~$50k/yr (1,300 lb/wk); a 20-25% 2nd-source slice = ~$12-19k/yr. Will that be attractive to each? Sizes are rough public estimates.</t>
+          <t>Sized for the SECOND-SOURCE slice: ~1 drum/week (~38 drums/yr), made FRESH each batch (18-day shelf life). Hard gates: (1) hold 90-95 C; (2) small/partial batches so you don't make more than the ~2 drums usable within 18 days.</t>
         </is>
       </c>
     </row>
@@ -1839,17 +1874,17 @@
       </c>
       <c r="B4" s="16" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Location</t>
         </is>
       </c>
       <c r="C4" s="16" t="inlineStr">
         <is>
-          <t>Location</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="D4" s="16" t="inlineStr">
         <is>
-          <t>Est. size</t>
+          <t>Holds 90-95 C?</t>
         </is>
       </c>
       <c r="E4" s="16" t="inlineStr">
@@ -1859,12 +1894,12 @@
       </c>
       <c r="F4" s="16" t="inlineStr">
         <is>
-          <t>Meets single-drum order?</t>
+          <t>Small-batch + 18-day fit</t>
         </is>
       </c>
       <c r="G4" s="16" t="inlineStr">
         <is>
-          <t>Small-acct fit</t>
+          <t>Volume feasibility</t>
         </is>
       </c>
       <c r="H4" s="16" t="inlineStr">
@@ -1874,44 +1909,9 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="29" t="inlineStr">
-        <is>
-          <t>SNP (incumbent)</t>
-        </is>
-      </c>
-      <c r="B5" s="29" t="inlineStr">
-        <is>
-          <t>Specialty chem / PVA maker</t>
-        </is>
-      </c>
-      <c r="C5" s="29" t="inlineStr">
-        <is>
-          <t>Durham, NC</t>
-        </is>
-      </c>
-      <c r="D5" s="29" t="inlineStr">
-        <is>
-          <t>~$4M, ~small</t>
-        </is>
-      </c>
-      <c r="E5" s="29" t="inlineStr">
-        <is>
-          <t>n/a (incumbent)</t>
-        </is>
-      </c>
-      <c r="F5" s="29" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G5" s="30" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="H5" s="29" t="inlineStr">
-        <is>
-          <t>PVA + alginates are core products; already your supplier. Best natural fit; main risk is small-vendor continuity.</t>
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>ACTIVE SHORTLIST — right-sized for ~1 drum/wk + 18-day shelf life</t>
         </is>
       </c>
     </row>
@@ -1923,528 +1923,669 @@
       </c>
       <c r="B6" s="29" t="inlineStr">
         <is>
-          <t>Coatings maker + contract mfg</t>
+          <t>Akron, OH</t>
         </is>
       </c>
       <c r="C6" s="29" t="inlineStr">
         <is>
-          <t>Akron, OH</t>
+          <t>▶ INTERVIEWING</t>
         </is>
       </c>
       <c r="D6" s="29" t="inlineStr">
         <is>
-          <t>~$28M, ~50-200 emp</t>
+          <t>Re-confirm (verbal yes earlier; list flags as gating)</t>
         </is>
       </c>
       <c r="E6" s="29" t="inlineStr">
         <is>
-          <t>100 gal (~2 drums)</t>
+          <t>from 5 gal</t>
         </is>
       </c>
       <c r="F6" s="29" t="inlineStr">
         <is>
-          <t>Below min for 1 drum; order 2-drum runs</t>
+          <t>Excellent — 5-gal floor easily makes 1 partial/full drum</t>
         </is>
       </c>
       <c r="G6" s="31" t="inlineStr">
         <is>
-          <t>Neutral / verify</t>
+          <t>GOOD</t>
         </is>
       </c>
       <c r="H6" s="29" t="inlineStr">
         <is>
-          <t>Confirmed 95C heating (gate cleared). 100-gal min batch + own product lines -&gt; may price single drums at a premium. STRONGEST new lead on capability.</t>
+          <t>Coatings house; pigment-dispersion specialty (good for your pigments); ISO 9001 / EPA-reg. CORRECTED: floor is ~5 gal, not 100. Gate to close in interview: 90-95 C hold.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="29" t="inlineStr">
         <is>
-          <t>ArroChem</t>
+          <t>CJB Applied Technologies</t>
         </is>
       </c>
       <c r="B7" s="29" t="inlineStr">
         <is>
-          <t>Family toll blender</t>
+          <t>Valdosta, GA</t>
         </is>
       </c>
       <c r="C7" s="29" t="inlineStr">
         <is>
-          <t>Mt Holly, NC</t>
+          <t>▶ INTERVIEWING (next call)</t>
         </is>
       </c>
       <c r="D7" s="29" t="inlineStr">
         <is>
-          <t>family-owned, 1 site</t>
+          <t>Confirm in interview</t>
         </is>
       </c>
       <c r="E7" s="29" t="inlineStr">
         <is>
-          <t>55 gal (1 drum)</t>
+          <t>3 pilot systems + small-batch + scale-up</t>
         </is>
       </c>
       <c r="F7" s="29" t="inlineStr">
         <is>
-          <t>Yes - exact match</t>
-        </is>
-      </c>
-      <c r="G7" s="30" t="inlineStr">
-        <is>
-          <t>Good (capability TBD)</t>
+          <t>Excellent — pilot plants, courts start-ups</t>
+        </is>
+      </c>
+      <c r="G7" s="31" t="inlineStr">
+        <is>
+          <t>GOOD</t>
         </is>
       </c>
       <c r="H7" s="29" t="inlineStr">
         <is>
-          <t>Advertised 55-5,000 gal batches = single drum is their floor. BUT failed trial: could not reach 95C. Re-confirm heating before relying on them.</t>
+          <t>Has an EX-LONZA (Proxel) formulator on staff — directly relevant to your biocide. (229) 588-7200.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="29" t="inlineStr">
         <is>
-          <t>Carolina Solvents</t>
+          <t>Piedmont Chemical</t>
         </is>
       </c>
       <c r="B8" s="29" t="inlineStr">
         <is>
-          <t>Small solvent/coating shop</t>
+          <t>High Point, NC</t>
         </is>
       </c>
       <c r="C8" s="29" t="inlineStr">
         <is>
-          <t>Hickory, NC</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D8" s="29" t="inlineStr">
         <is>
-          <t>&lt;$5M, &lt;25 emp</t>
+          <t>Confirm 90-95 C</t>
         </is>
       </c>
       <c r="E8" s="29" t="inlineStr">
         <is>
-          <t>unknown (small)</t>
+          <t>pilot reactors 5-100 gal</t>
         </is>
       </c>
       <c r="F8" s="29" t="inlineStr">
         <is>
-          <t>Likely yes</t>
-        </is>
-      </c>
-      <c r="G8" s="30" t="inlineStr">
-        <is>
-          <t>Good / verify process</t>
+          <t>Good — 5-gal floor fits a single drum</t>
+        </is>
+      </c>
+      <c r="G8" s="31" t="inlineStr">
+        <is>
+          <t>GOOD</t>
         </is>
       </c>
       <c r="H8" s="29" t="inlineStr">
         <is>
-          <t>Smallest -&gt; would value the account. Solvent/ambient focus; CONFIRM heated aqueous 95C capability. Not yet contacted.</t>
+          <t>UPGRADED from earlier 'too big': textile/PVA heritage = real PVA know-how; family-owned/agile. Best blend of PVA expertise + small-batch fit. (336) 885-5131.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="29" t="inlineStr">
         <is>
-          <t>Piedmont Chemical</t>
+          <t>Columbus Chemical (CCI)</t>
         </is>
       </c>
       <c r="B9" s="29" t="inlineStr">
         <is>
-          <t>Custom synthesis/polymer</t>
+          <t>Columbus, WI / Phoenix, AZ</t>
         </is>
       </c>
       <c r="C9" s="29" t="inlineStr">
         <is>
-          <t>High Point, NC</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D9" s="29" t="inlineStr">
         <is>
-          <t>~$35M, ~64-180 emp</t>
+          <t>Yes — heating/cooling</t>
         </is>
       </c>
       <c r="E9" s="29" t="inlineStr">
         <is>
-          <t>unknown (larger)</t>
+          <t>20 L - 20,000 L (~5 gal floor)</t>
         </is>
       </c>
       <c r="F9" s="29" t="inlineStr">
         <is>
-          <t>Probably below their sweet spot</t>
-        </is>
-      </c>
-      <c r="G9" s="31" t="inlineStr">
-        <is>
-          <t>Caution / lean too big</t>
+          <t>Excellent — lowest floor, widest range</t>
+        </is>
+      </c>
+      <c r="G9" s="32" t="inlineStr">
+        <is>
+          <t>STRONG</t>
         </is>
       </c>
       <c r="H9" s="29" t="inlineStr">
         <is>
-          <t>Synthesis orientation wants bigger campaigns; a single-drum blend likely under-prioritized or premium-priced.</t>
+          <t>In-house lab, ISO 9001. Widest batch range = least shelf-life waste; can scale if demand grows.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="29" t="inlineStr">
         <is>
-          <t>ILC Dover</t>
+          <t>CORECHEM</t>
         </is>
       </c>
       <c r="B10" s="29" t="inlineStr">
         <is>
-          <t>Pharma/aerospace (Ingersoll Rand)</t>
+          <t>Knoxville, TN</t>
         </is>
       </c>
       <c r="C10" s="29" t="inlineStr">
         <is>
-          <t>Frederica, DE</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="D10" s="29" t="inlineStr">
         <is>
-          <t>$80M-$450M, ~2,100 emp</t>
+          <t>Confirm</t>
         </is>
       </c>
       <c r="E10" s="29" t="inlineStr">
         <is>
-          <t>n/a - equipment/services</t>
+          <t>smallest tank ~250 gal (~4.5 drums)</t>
         </is>
       </c>
       <c r="F10" s="29" t="inlineStr">
         <is>
-          <t>No - wrong category</t>
-        </is>
-      </c>
-      <c r="G10" s="32" t="inlineStr">
-        <is>
-          <t>Too big / wrong type</t>
+          <t>CAUTION — 250-gal min may overshoot 18-day shelf life</t>
+        </is>
+      </c>
+      <c r="G10" s="33" t="inlineStr">
+        <is>
+          <t>CAUTION</t>
         </is>
       </c>
       <c r="H10" s="29" t="inlineStr">
         <is>
-          <t>Could NOT reach 95C and is an equipment/containment firm, not a drum toll blender. Recommend deprioritize/close out.</t>
+          <t>Low-MOQ, start-up-friendly, family-owned. ASK about PARTIAL batches: a full 250-gal batch = ~4.5 drums but you can only use ~2 within 18 days.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>Northstar Chemical</t>
+        </is>
+      </c>
+      <c r="B11" s="29" t="inlineStr">
+        <is>
+          <t>Charlotte, NC</t>
+        </is>
+      </c>
+      <c r="C11" s="29" t="inlineStr">
+        <is>
+          <t>Backup</t>
+        </is>
+      </c>
+      <c r="D11" s="29" t="inlineStr">
+        <is>
+          <t>Confirm</t>
+        </is>
+      </c>
+      <c r="E11" s="29" t="inlineStr">
+        <is>
+          <t>unknown (small custom/toll)</t>
+        </is>
+      </c>
+      <c r="F11" s="29" t="inlineStr">
+        <is>
+          <t>Likely good — verify</t>
+        </is>
+      </c>
+      <c r="G11" s="31" t="inlineStr">
+        <is>
+          <t>LIKELY GOOD</t>
+        </is>
+      </c>
+      <c r="H11" s="29" t="inlineStr">
+        <is>
+          <t>Smaller dry-to-liquid custom/toll blender. (800) 570-0204.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>RESIN SUPPLIERS &amp; DISTRIBUTORS (raw PVA, not toll-blended solution)</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n"/>
-      <c r="F12" s="3" t="n"/>
-      <c r="G12" s="3" t="n"/>
-      <c r="H12" s="3" t="n"/>
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>TECHNICAL ADVISOR — won't supply at this volume, but free expert call</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="29" t="inlineStr">
         <is>
-          <t>Brenntag</t>
+          <t>Sekisui Specialty Chemicals</t>
         </is>
       </c>
       <c r="B13" s="29" t="inlineStr">
         <is>
-          <t>World's largest chem distributor</t>
+          <t>Calvert City, KY / Pasadena, TX</t>
         </is>
       </c>
       <c r="C13" s="29" t="inlineStr">
         <is>
-          <t>Essen, DE / US-wide</t>
+          <t>Advisor only</t>
         </is>
       </c>
       <c r="D13" s="29" t="inlineStr">
         <is>
-          <t>~EUR15B, ~17k emp</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="E13" s="29" t="inlineStr">
         <is>
-          <t>single drums (core)</t>
+          <t>n/a (producer, bulk only)</t>
         </is>
       </c>
       <c r="F13" s="29" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G13" s="31" t="inlineStr">
-        <is>
-          <t>Neutral (serve, no VIP)</t>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G13" s="34" t="inlineStr">
+        <is>
+          <t>N/A — advisor</t>
         </is>
       </c>
       <c r="H13" s="29" t="inlineStr">
         <is>
-          <t>Already lists Sekisui Selvol PVA -&gt; easiest source of genuine resin in drums. You'll be a small/transactional account; possible small-order premium.</t>
+          <t>Largest US PVOH (Selvol) producer. Free Tech Services call on grade selection + cook procedure. +1 855 436 8683.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="29" t="inlineStr">
-        <is>
-          <t>Tilley Distribution</t>
-        </is>
-      </c>
-      <c r="B14" s="29" t="inlineStr">
-        <is>
-          <t>Regional specialty distributor (PE-backed)</t>
-        </is>
-      </c>
-      <c r="C14" s="29" t="inlineStr">
-        <is>
-          <t>Baltimore, MD</t>
-        </is>
-      </c>
-      <c r="D14" s="29" t="inlineStr">
-        <is>
-          <t>~$40M, ~120-180 emp</t>
-        </is>
-      </c>
-      <c r="E14" s="29" t="inlineStr">
-        <is>
-          <t>drums/small lots</t>
-        </is>
-      </c>
-      <c r="F14" s="29" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G14" s="30" t="inlineStr">
-        <is>
-          <t>Good (best relationship fit)</t>
-        </is>
-      </c>
-      <c r="H14" s="29" t="inlineStr">
-        <is>
-          <t>$25k account is meaningful to them; relationship-oriented. OPEN: confirm they actually source a PVA brand. Was already flagged as slow/maybe can't meet.</t>
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>DROPPED — too large / MOQ mismatch for ~1 drum/wk</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="29" t="inlineStr">
         <is>
-          <t>Palmer Holland</t>
+          <t>Goulston Technologies</t>
         </is>
       </c>
       <c r="B15" s="29" t="inlineStr">
         <is>
-          <t>Mid-size NA distributor (ESOP)</t>
+          <t>Monroe, NC</t>
         </is>
       </c>
       <c r="C15" s="29" t="inlineStr">
         <is>
-          <t>Westlake, OH</t>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="D15" s="29" t="inlineStr">
         <is>
-          <t>~250 emp, national</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E15" s="29" t="inlineStr">
         <is>
-          <t>drums/specialty lots</t>
+          <t>large</t>
         </is>
       </c>
       <c r="F15" s="29" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G15" s="30" t="inlineStr">
-        <is>
-          <t>Good-Neutral</t>
+          <t>Too big</t>
+        </is>
+      </c>
+      <c r="G15" s="35" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="H15" s="29" t="inlineStr">
         <is>
-          <t>Employee-owned, relationship-driven, workable size. OPEN: confirm they carry a PVA principal (unverified).</t>
+          <t>Large textile chemical maker. 704-289-6464.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="29" t="inlineStr">
         <is>
-          <t>Barentz</t>
+          <t>3V Sigma USA</t>
         </is>
       </c>
       <c r="B16" s="29" t="inlineStr">
         <is>
-          <t>Large global specialty distributor</t>
+          <t>Georgetown, SC</t>
         </is>
       </c>
       <c r="C16" s="29" t="inlineStr">
         <is>
-          <t>Hoofddorp, NL / NA</t>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="D16" s="29" t="inlineStr">
         <is>
-          <t>~EUR2.4B, ~2,700 emp</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E16" s="29" t="inlineStr">
         <is>
-          <t>drums (focus skews large)</t>
+          <t>large</t>
         </is>
       </c>
       <c r="F16" s="29" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G16" s="32" t="inlineStr">
-        <is>
-          <t>Likely too big to prioritize</t>
+          <t>Too big</t>
+        </is>
+      </c>
+      <c r="G16" s="35" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="H16" s="29" t="inlineStr">
         <is>
-          <t>Lists PVA and can serve, but a tiny industrial-drum account isn't their priority segment.</t>
+          <t>Large specialty chemical producer.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="29" t="inlineStr">
         <is>
-          <t>Sekisui Specialty Chem</t>
+          <t>Royal Chemical</t>
         </is>
       </c>
       <c r="B17" s="29" t="inlineStr">
         <is>
-          <t>PVA PRODUCER (Selvol)</t>
+          <t>Twinsburg, OH (+5 sites)</t>
         </is>
       </c>
       <c r="C17" s="29" t="inlineStr">
         <is>
-          <t>Dallas, TX</t>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="D17" s="29" t="inlineStr">
         <is>
-          <t>~$186M US, ~260-400 emp</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E17" s="29" t="inlineStr">
         <is>
-          <t>bulk; NOT direct</t>
+          <t>220-gal liquid MOQ (~4 drums)</t>
         </is>
       </c>
       <c r="F17" s="29" t="inlineStr">
         <is>
-          <t>No (via distributor)</t>
-        </is>
-      </c>
-      <c r="G17" s="32" t="inlineStr">
-        <is>
-          <t>Too small to buy direct</t>
+          <t>MOQ overshoots shelf life</t>
+        </is>
+      </c>
+      <c r="G17" s="35" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="H17" s="29" t="inlineStr">
         <is>
-          <t>It IS Selvol (your reference resin). Won't sell factory-direct at your volume -&gt; routes you to Brenntag etc.</t>
+          <t>220-gal min = ~4 drums = ~4 wks supply &gt; 18-day shelf life.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="29" t="inlineStr">
         <is>
-          <t>Kuraray</t>
+          <t>Columbia Chemical</t>
         </is>
       </c>
       <c r="B18" s="29" t="inlineStr">
         <is>
-          <t>World's largest PVA PRODUCER</t>
+          <t>Brunswick, OH</t>
         </is>
       </c>
       <c r="C18" s="29" t="inlineStr">
         <is>
-          <t>Tokyo / Houston TX</t>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="D18" s="29" t="inlineStr">
         <is>
-          <t>~$5.4B, ~12k emp</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E18" s="29" t="inlineStr">
         <is>
-          <t>bulk; NOT direct</t>
+          <t>large</t>
         </is>
       </c>
       <c r="F18" s="29" t="inlineStr">
         <is>
-          <t>No (via distributor)</t>
-        </is>
-      </c>
-      <c r="G18" s="32" t="inlineStr">
-        <is>
-          <t>Too small to buy direct</t>
-        </is>
-      </c>
-      <c r="H18" s="29" t="inlineStr">
-        <is>
-          <t>Poval/Elvanol brand owner. Buy via named distributors: dar-tech (Buffalo NY, closest East Coast) or Associated Agencies.</t>
-        </is>
-      </c>
+          <t>Too big / mismatch</t>
+        </is>
+      </c>
+      <c r="G18" s="35" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H18" s="29" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="29" t="inlineStr">
-        <is>
-          <t>Aldon Corp</t>
-        </is>
-      </c>
-      <c r="B19" s="29" t="inlineStr">
-        <is>
-          <t>Lab/education chem + contract blender</t>
-        </is>
-      </c>
-      <c r="C19" s="29" t="inlineStr">
-        <is>
-          <t>Avon, NY</t>
-        </is>
-      </c>
-      <c r="D19" s="29" t="inlineStr">
-        <is>
-          <t>small, private</t>
-        </is>
-      </c>
-      <c r="E19" s="29" t="inlineStr">
-        <is>
-          <t>lab bottles, not drums</t>
-        </is>
-      </c>
-      <c r="F19" s="29" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G19" s="32" t="inlineStr">
-        <is>
-          <t>Poor / wrong type</t>
-        </is>
-      </c>
-      <c r="H19" s="29" t="inlineStr">
-        <is>
-          <t>Education &amp; private-label LAB-grade PVA solutions only. Not an industrial drum-resin source. Close out.</t>
+      <c r="A19" s="30" t="inlineStr">
+        <is>
+          <t>ELIMINATED — failed the 90-95 C cook</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="29" t="inlineStr">
+        <is>
+          <t>ArroChem</t>
+        </is>
+      </c>
+      <c r="B20" s="29" t="inlineStr">
+        <is>
+          <t>Mt. Holly, NC</t>
+        </is>
+      </c>
+      <c r="C20" s="29" t="inlineStr">
+        <is>
+          <t>ELIMINATED</t>
+        </is>
+      </c>
+      <c r="D20" s="29" t="inlineStr">
+        <is>
+          <t>85 C ceiling — FAILS</t>
+        </is>
+      </c>
+      <c r="E20" s="29" t="inlineStr">
+        <is>
+          <t>55 gal (would have fit)</t>
+        </is>
+      </c>
+      <c r="F20" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G20" s="35" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H20" s="29" t="inlineStr">
+        <is>
+          <t>Volume fit was perfect (55-gal floor) but can't reach the 90-95 C cook.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>NOTE: Producers (Sekisui, Kuraray) won't sell direct at this volume -&gt; go through a distributor. Brenntag already stocks Selvol. Distributors supply RAW RESIN; you still need a toll blender (top section) to make the liquid solution.</t>
+      <c r="A21" s="29" t="inlineStr">
+        <is>
+          <t>ILC Dover</t>
+        </is>
+      </c>
+      <c r="B21" s="29" t="inlineStr">
+        <is>
+          <t>Frederica, DE</t>
+        </is>
+      </c>
+      <c r="C21" s="29" t="inlineStr">
+        <is>
+          <t>ELIMINATED</t>
+        </is>
+      </c>
+      <c r="D21" s="29" t="inlineStr">
+        <is>
+          <t>Can't reach 95 C</t>
+        </is>
+      </c>
+      <c r="E21" s="29" t="inlineStr">
+        <is>
+          <t>n/a (equipment firm)</t>
+        </is>
+      </c>
+      <c r="F21" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G21" s="35" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H21" s="29" t="inlineStr">
+        <is>
+          <t>Wrong category (Ingersoll Rand containment/equipment) + heating fail. Close out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="30" t="inlineStr">
+        <is>
+          <t>RAW RESIN PATH — reference only (supply Selvol resin, not the liquid blend)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="29" t="inlineStr">
+        <is>
+          <t>Brenntag</t>
+        </is>
+      </c>
+      <c r="B23" s="29" t="inlineStr">
+        <is>
+          <t>US-wide</t>
+        </is>
+      </c>
+      <c r="C23" s="29" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="D23" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E23" s="29" t="inlineStr">
+        <is>
+          <t>single drums (core)</t>
+        </is>
+      </c>
+      <c r="F23" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G23" s="34" t="inlineStr">
+        <is>
+          <t>N/A — distributor</t>
+        </is>
+      </c>
+      <c r="H23" s="29" t="inlineStr">
+        <is>
+          <t>Already lists Sekisui Selvol → easiest source of genuine resin in drums if a blender needs it supplied.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="29" t="inlineStr">
+        <is>
+          <t>Tilley / Palmer Holland</t>
+        </is>
+      </c>
+      <c r="B24" s="29" t="inlineStr">
+        <is>
+          <t>Baltimore, MD / Westlake, OH</t>
+        </is>
+      </c>
+      <c r="C24" s="29" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="D24" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E24" s="29" t="inlineStr">
+        <is>
+          <t>drums</t>
+        </is>
+      </c>
+      <c r="F24" s="29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G24" s="34" t="inlineStr">
+        <is>
+          <t>N/A — distributor</t>
+        </is>
+      </c>
+      <c r="H24" s="29" t="inlineStr">
+        <is>
+          <t>Relationship-sized distributors; confirm they carry a PVA brand. Use only if sourcing raw resin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Legend: STRONG/GOOD = green, CAUTION/LIKELY = amber, NO = red, advisor/distributor = grey. 'Holds 90-95 C?' is the hard gate — re-confirm in every interview.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A21:H21"/>
+  <mergeCells count="8">
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A26:H26"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A22:H22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>